<commit_message>
Complete Habrit Khadasha Structure
EH'YEH ASHER EH'YEH
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -18,30 +18,36 @@
     <t>Seh HaElohim</t>
   </si>
   <si>
+    <t>She'Elohim</t>
+  </si>
+  <si>
+    <t>HaElohim</t>
+  </si>
+  <si>
+    <t>L'Elohim</t>
+  </si>
+  <si>
+    <t>Elohecha</t>
+  </si>
+  <si>
+    <t>HaElohim Moshi’enu</t>
+  </si>
+  <si>
+    <t>Hesed HaElohim</t>
+  </si>
+  <si>
     <t>Peter</t>
   </si>
   <si>
-    <t>She'Elohim</t>
-  </si>
-  <si>
     <t>Kefa</t>
   </si>
   <si>
-    <t>HaElohim</t>
-  </si>
-  <si>
     <t>Judea</t>
   </si>
   <si>
-    <t>L'Elohim</t>
-  </si>
-  <si>
     <t>Y'udah</t>
   </si>
   <si>
-    <t>Elohecha</t>
-  </si>
-  <si>
     <t>John</t>
   </si>
   <si>
@@ -54,15 +60,9 @@
     <t>Yerushalayim</t>
   </si>
   <si>
-    <t>HaElohim Moshi’enu</t>
-  </si>
-  <si>
     <t>James</t>
   </si>
   <si>
-    <t>Hesed HaElohim</t>
-  </si>
-  <si>
     <t>Yakov</t>
   </si>
   <si>
@@ -147,6 +147,9 @@
     <t>Isaac</t>
   </si>
   <si>
+    <t>עברית</t>
+  </si>
+  <si>
     <t>Yitzhak</t>
   </si>
   <si>
@@ -156,9 +159,6 @@
     <t>Avraham</t>
   </si>
   <si>
-    <t>עברית</t>
-  </si>
-  <si>
     <t>Judah</t>
   </si>
   <si>
@@ -195,6 +195,9 @@
     <t>Paul</t>
   </si>
   <si>
+    <t>한국</t>
+  </si>
+  <si>
     <t>Sha'ul</t>
   </si>
   <si>
@@ -211,9 +214,6 @@
   </si>
   <si>
     <t>Joshua</t>
-  </si>
-  <si>
-    <t>한국</t>
   </si>
   <si>
     <t>English</t>
@@ -585,10 +585,10 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>67</v>
@@ -636,32 +636,32 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -678,35 +678,35 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
@@ -809,15 +809,15 @@
         <v>43</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13">
@@ -825,7 +825,7 @@
         <v>48</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -873,28 +873,28 @@
         <v>59</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EH'YEH to Bereshit - Start Shemot
Copy in all verses for the book Bereshit
Fix Footer for some files.... not all
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -13,68 +13,71 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="74">
+  <si>
+    <t>Peter</t>
+  </si>
   <si>
     <t>Seh HaElohim</t>
   </si>
   <si>
+    <t>Kefa</t>
+  </si>
+  <si>
+    <t>Judea</t>
+  </si>
+  <si>
     <t>She'Elohim</t>
   </si>
   <si>
+    <t>Y'udah</t>
+  </si>
+  <si>
     <t>HaElohim</t>
   </si>
   <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Yochanan</t>
+  </si>
+  <si>
     <t>L'Elohim</t>
   </si>
   <si>
+    <t>Jerusalem</t>
+  </si>
+  <si>
+    <t>Yerushalayim</t>
+  </si>
+  <si>
     <t>Elohecha</t>
   </si>
   <si>
+    <t>James</t>
+  </si>
+  <si>
+    <t>Yakov</t>
+  </si>
+  <si>
     <t>HaElohim Moshi’enu</t>
   </si>
   <si>
+    <t>Mount of Olives</t>
+  </si>
+  <si>
+    <t>Har Ha-Zeitim</t>
+  </si>
+  <si>
     <t>Hesed HaElohim</t>
   </si>
   <si>
-    <t>Peter</t>
-  </si>
-  <si>
-    <t>Kefa</t>
-  </si>
-  <si>
-    <t>Judea</t>
-  </si>
-  <si>
-    <t>Y'udah</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Yochanan</t>
-  </si>
-  <si>
-    <t>Jerusalem</t>
-  </si>
-  <si>
-    <t>Yerushalayim</t>
-  </si>
-  <si>
-    <t>James</t>
-  </si>
-  <si>
-    <t>Yakov</t>
-  </si>
-  <si>
-    <t>Mount of Olives</t>
-  </si>
-  <si>
-    <t>Har Ha-Zeitim</t>
-  </si>
-  <si>
     <t>Mary</t>
   </si>
   <si>
+    <t>El Roi</t>
+  </si>
+  <si>
     <t>Miriam</t>
   </si>
   <si>
@@ -147,73 +150,73 @@
     <t>Isaac</t>
   </si>
   <si>
+    <t>Yitzhak</t>
+  </si>
+  <si>
+    <t>Abraham</t>
+  </si>
+  <si>
+    <t>Avraham</t>
+  </si>
+  <si>
+    <t>Judah</t>
+  </si>
+  <si>
+    <t>Simon</t>
+  </si>
+  <si>
+    <t>Shimon</t>
+  </si>
+  <si>
+    <t>Pilate</t>
+  </si>
+  <si>
+    <t>Pilatos</t>
+  </si>
+  <si>
+    <t>Caesar</t>
+  </si>
+  <si>
+    <t>Keisar</t>
+  </si>
+  <si>
+    <t>Joanna</t>
+  </si>
+  <si>
+    <t>Yochana</t>
+  </si>
+  <si>
+    <t>Cloepas</t>
+  </si>
+  <si>
+    <t>Cleofas</t>
+  </si>
+  <si>
+    <t>Paul</t>
+  </si>
+  <si>
+    <t>Sha'ul</t>
+  </si>
+  <si>
+    <t>Herod</t>
+  </si>
+  <si>
+    <t>Hordos</t>
+  </si>
+  <si>
+    <t>Timothy</t>
+  </si>
+  <si>
+    <t>Timotheos</t>
+  </si>
+  <si>
+    <t>Joshua</t>
+  </si>
+  <si>
     <t>עברית</t>
   </si>
   <si>
-    <t>Yitzhak</t>
-  </si>
-  <si>
-    <t>Abraham</t>
-  </si>
-  <si>
-    <t>Avraham</t>
-  </si>
-  <si>
-    <t>Judah</t>
-  </si>
-  <si>
-    <t>Simon</t>
-  </si>
-  <si>
-    <t>Shimon</t>
-  </si>
-  <si>
-    <t>Pilate</t>
-  </si>
-  <si>
-    <t>Pilatos</t>
-  </si>
-  <si>
-    <t>Caesar</t>
-  </si>
-  <si>
-    <t>Keisar</t>
-  </si>
-  <si>
-    <t>Joanna</t>
-  </si>
-  <si>
-    <t>Yochana</t>
-  </si>
-  <si>
-    <t>Cloepas</t>
-  </si>
-  <si>
-    <t>Cleofas</t>
-  </si>
-  <si>
-    <t>Paul</t>
-  </si>
-  <si>
     <t>한국</t>
-  </si>
-  <si>
-    <t>Sha'ul</t>
-  </si>
-  <si>
-    <t>Herod</t>
-  </si>
-  <si>
-    <t>Hordos</t>
-  </si>
-  <si>
-    <t>Timothy</t>
-  </si>
-  <si>
-    <t>Timotheos</t>
-  </si>
-  <si>
-    <t>Joshua</t>
   </si>
   <si>
     <t>English</t>
@@ -585,30 +588,30 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -631,37 +634,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -678,44 +686,44 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -723,90 +731,90 @@
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>45</v>
@@ -825,7 +833,7 @@
         <v>48</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -873,28 +881,28 @@
         <v>59</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjust all word doc Footers
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -15,43 +15,49 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="74">
   <si>
+    <t>Seh HaElohim</t>
+  </si>
+  <si>
     <t>Peter</t>
   </si>
   <si>
-    <t>Seh HaElohim</t>
-  </si>
-  <si>
     <t>Kefa</t>
   </si>
   <si>
+    <t>She'Elohim</t>
+  </si>
+  <si>
     <t>Judea</t>
   </si>
   <si>
-    <t>She'Elohim</t>
+    <t>HaElohim</t>
   </si>
   <si>
     <t>Y'udah</t>
   </si>
   <si>
-    <t>HaElohim</t>
+    <t>L'Elohim</t>
   </si>
   <si>
     <t>John</t>
   </si>
   <si>
+    <t>Elohecha</t>
+  </si>
+  <si>
     <t>Yochanan</t>
   </si>
   <si>
-    <t>L'Elohim</t>
-  </si>
-  <si>
     <t>Jerusalem</t>
   </si>
   <si>
+    <t>HaElohim Moshi’enu</t>
+  </si>
+  <si>
     <t>Yerushalayim</t>
   </si>
   <si>
-    <t>Elohecha</t>
+    <t>Hesed HaElohim</t>
   </si>
   <si>
     <t>James</t>
@@ -60,7 +66,7 @@
     <t>Yakov</t>
   </si>
   <si>
-    <t>HaElohim Moshi’enu</t>
+    <t>El Roi</t>
   </si>
   <si>
     <t>Mount of Olives</t>
@@ -69,13 +75,7 @@
     <t>Har Ha-Zeitim</t>
   </si>
   <si>
-    <t>Hesed HaElohim</t>
-  </si>
-  <si>
     <t>Mary</t>
-  </si>
-  <si>
-    <t>El Roi</t>
   </si>
   <si>
     <t>Miriam</t>
@@ -634,42 +634,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -686,49 +686,49 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>21</v>
@@ -833,7 +833,7 @@
         <v>48</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Finish First upload of Shemot
EH'YEH ASHER EH'YEH
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -21,54 +21,54 @@
     <t>Peter</t>
   </si>
   <si>
+    <t>She'Elohim</t>
+  </si>
+  <si>
+    <t>HaElohim</t>
+  </si>
+  <si>
+    <t>L'Elohim</t>
+  </si>
+  <si>
+    <t>Elohecha</t>
+  </si>
+  <si>
     <t>Kefa</t>
   </si>
   <si>
-    <t>She'Elohim</t>
+    <t>HaElohim Moshi’enu</t>
+  </si>
+  <si>
+    <t>Hesed HaElohim</t>
   </si>
   <si>
     <t>Judea</t>
   </si>
   <si>
-    <t>HaElohim</t>
+    <t>El Roi</t>
   </si>
   <si>
     <t>Y'udah</t>
   </si>
   <si>
-    <t>L'Elohim</t>
-  </si>
-  <si>
     <t>John</t>
   </si>
   <si>
-    <t>Elohecha</t>
-  </si>
-  <si>
     <t>Yochanan</t>
   </si>
   <si>
     <t>Jerusalem</t>
   </si>
   <si>
-    <t>HaElohim Moshi’enu</t>
-  </si>
-  <si>
     <t>Yerushalayim</t>
   </si>
   <si>
-    <t>Hesed HaElohim</t>
-  </si>
-  <si>
     <t>James</t>
   </si>
   <si>
     <t>Yakov</t>
   </si>
   <si>
-    <t>El Roi</t>
-  </si>
-  <si>
     <t>Mount of Olives</t>
   </si>
   <si>
@@ -168,6 +168,9 @@
     <t>Shimon</t>
   </si>
   <si>
+    <t>עברית</t>
+  </si>
+  <si>
     <t>Pilate</t>
   </si>
   <si>
@@ -211,9 +214,6 @@
   </si>
   <si>
     <t>Joshua</t>
-  </si>
-  <si>
-    <t>עברית</t>
   </si>
   <si>
     <t>한국</t>
@@ -588,7 +588,7 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>67</v>
@@ -639,37 +639,37 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -689,35 +689,35 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>18</v>
@@ -833,7 +833,7 @@
         <v>48</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -846,63 +846,63 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove ' from EHYEH, finish Shoftim structure
EHYEH ASHER EHYEH
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -4,8 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Names of Adonai" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Names of People" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Names of People" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -13,41 +12,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="74">
-  <si>
-    <t>Seh HaElohim</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="65">
   <si>
     <t>Peter</t>
   </si>
   <si>
-    <t>She'Elohim</t>
-  </si>
-  <si>
-    <t>HaElohim</t>
-  </si>
-  <si>
-    <t>L'Elohim</t>
-  </si>
-  <si>
-    <t>Elohecha</t>
-  </si>
-  <si>
     <t>Kefa</t>
   </si>
   <si>
-    <t>HaElohim Moshi’enu</t>
-  </si>
-  <si>
-    <t>Hesed HaElohim</t>
-  </si>
-  <si>
     <t>Judea</t>
   </si>
   <si>
-    <t>El Roi</t>
-  </si>
-  <si>
     <t>Y'udah</t>
   </si>
   <si>
@@ -168,54 +143,54 @@
     <t>Shimon</t>
   </si>
   <si>
+    <t>Pilate</t>
+  </si>
+  <si>
+    <t>Pilatos</t>
+  </si>
+  <si>
+    <t>Caesar</t>
+  </si>
+  <si>
+    <t>Keisar</t>
+  </si>
+  <si>
+    <t>Joanna</t>
+  </si>
+  <si>
+    <t>Yochana</t>
+  </si>
+  <si>
+    <t>Cloepas</t>
+  </si>
+  <si>
+    <t>Cleofas</t>
+  </si>
+  <si>
+    <t>Paul</t>
+  </si>
+  <si>
+    <t>Sha'ul</t>
+  </si>
+  <si>
+    <t>Herod</t>
+  </si>
+  <si>
+    <t>Hordos</t>
+  </si>
+  <si>
+    <t>Timothy</t>
+  </si>
+  <si>
+    <t>Timotheos</t>
+  </si>
+  <si>
+    <t>Joshua</t>
+  </si>
+  <si>
     <t>עברית</t>
   </si>
   <si>
-    <t>Pilate</t>
-  </si>
-  <si>
-    <t>Pilatos</t>
-  </si>
-  <si>
-    <t>Caesar</t>
-  </si>
-  <si>
-    <t>Keisar</t>
-  </si>
-  <si>
-    <t>Joanna</t>
-  </si>
-  <si>
-    <t>Yochana</t>
-  </si>
-  <si>
-    <t>Cloepas</t>
-  </si>
-  <si>
-    <t>Cleofas</t>
-  </si>
-  <si>
-    <t>Paul</t>
-  </si>
-  <si>
-    <t>Sha'ul</t>
-  </si>
-  <si>
-    <t>Herod</t>
-  </si>
-  <si>
-    <t>Hordos</t>
-  </si>
-  <si>
-    <t>Timothy</t>
-  </si>
-  <si>
-    <t>Timotheos</t>
-  </si>
-  <si>
-    <t>Joshua</t>
-  </si>
-  <si>
     <t>한국</t>
   </si>
   <si>
@@ -232,9 +207,6 @@
   </si>
   <si>
     <t>YIHOVEH</t>
-  </si>
-  <si>
-    <t>YHWH</t>
   </si>
 </sst>
 </file>
@@ -362,10 +334,6 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -588,30 +556,30 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -623,61 +591,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="17.63"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -686,223 +599,223 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Structure for Shmuel 1 uploaded
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -140,6 +140,9 @@
     <t>Simon</t>
   </si>
   <si>
+    <t>עברית</t>
+  </si>
+  <si>
     <t>Shimon</t>
   </si>
   <si>
@@ -186,9 +189,6 @@
   </si>
   <si>
     <t>Joshua</t>
-  </si>
-  <si>
-    <t>עברית</t>
   </si>
   <si>
     <t>한국</t>
@@ -556,7 +556,7 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>59</v>
@@ -754,68 +754,68 @@
         <v>41</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Total Structure Revamp -- 45 Books
EHYEH ASHER EHYEH
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -140,55 +140,55 @@
     <t>Simon</t>
   </si>
   <si>
+    <t>Shimon</t>
+  </si>
+  <si>
+    <t>Pilate</t>
+  </si>
+  <si>
+    <t>Pilatos</t>
+  </si>
+  <si>
+    <t>Caesar</t>
+  </si>
+  <si>
+    <t>Keisar</t>
+  </si>
+  <si>
+    <t>Joanna</t>
+  </si>
+  <si>
+    <t>Yochana</t>
+  </si>
+  <si>
+    <t>Cloepas</t>
+  </si>
+  <si>
+    <t>Cleofas</t>
+  </si>
+  <si>
+    <t>Paul</t>
+  </si>
+  <si>
+    <t>Sha'ul</t>
+  </si>
+  <si>
+    <t>Herod</t>
+  </si>
+  <si>
+    <t>Hordos</t>
+  </si>
+  <si>
+    <t>Timothy</t>
+  </si>
+  <si>
+    <t>Timotheos</t>
+  </si>
+  <si>
+    <t>Joshua</t>
+  </si>
+  <si>
     <t>עברית</t>
-  </si>
-  <si>
-    <t>Shimon</t>
-  </si>
-  <si>
-    <t>Pilate</t>
-  </si>
-  <si>
-    <t>Pilatos</t>
-  </si>
-  <si>
-    <t>Caesar</t>
-  </si>
-  <si>
-    <t>Keisar</t>
-  </si>
-  <si>
-    <t>Joanna</t>
-  </si>
-  <si>
-    <t>Yochana</t>
-  </si>
-  <si>
-    <t>Cloepas</t>
-  </si>
-  <si>
-    <t>Cleofas</t>
-  </si>
-  <si>
-    <t>Paul</t>
-  </si>
-  <si>
-    <t>Sha'ul</t>
-  </si>
-  <si>
-    <t>Herod</t>
-  </si>
-  <si>
-    <t>Hordos</t>
-  </si>
-  <si>
-    <t>Timothy</t>
-  </si>
-  <si>
-    <t>Timotheos</t>
-  </si>
-  <si>
-    <t>Joshua</t>
   </si>
   <si>
     <t>한국</t>
@@ -556,7 +556,7 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>59</v>
@@ -754,68 +754,68 @@
         <v>41</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>